<commit_message>
removed format 96 variables froom lookup table
</commit_message>
<xml_diff>
--- a/lookup.xlsx
+++ b/lookup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asacarny/Repositories/hospital-cost-reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64aef9a73715520e/Documents/projects/hospital-cost-reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA14F41D-D4A4-0641-AA77-13E05DC77C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{BA14F41D-D4A4-0641-AA77-13E05DC77C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDC5F117-9B00-4ABC-AFF2-B2E6BC5FC0D5}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="500" windowWidth="13080" windowHeight="19860" xr2:uid="{2FC29EAB-8935-714F-80E4-2DC39A71C1EE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{2FC29EAB-8935-714F-80E4-2DC39A71C1EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup Table" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="151">
   <si>
     <t>rec</t>
   </si>
@@ -203,30 +203,12 @@
     <t>01400</t>
   </si>
   <si>
-    <t>0100</t>
-  </si>
-  <si>
     <t>00900</t>
   </si>
   <si>
-    <t>0200</t>
-  </si>
-  <si>
-    <t>0300</t>
-  </si>
-  <si>
-    <t>02400</t>
-  </si>
-  <si>
     <t>chguccare</t>
   </si>
   <si>
-    <t>0600</t>
-  </si>
-  <si>
-    <t>1500</t>
-  </si>
-  <si>
     <t>00500</t>
   </si>
   <si>
@@ -266,12 +248,6 @@
     <t>02900</t>
   </si>
   <si>
-    <t>costuccare</t>
-  </si>
-  <si>
-    <t>03100</t>
-  </si>
-  <si>
     <t>beds - adults &amp; peds</t>
   </si>
   <si>
@@ -401,9 +377,6 @@
     <t>other special care beds</t>
   </si>
   <si>
-    <t>02140</t>
-  </si>
-  <si>
     <t>non-medicare bad debt expense (2010 format only)</t>
   </si>
   <si>
@@ -446,66 +419,12 @@
     <t>prog_net_chg</t>
   </si>
   <si>
-    <t>0500</t>
-  </si>
-  <si>
-    <t>D40A180</t>
-  </si>
-  <si>
-    <t>10300</t>
-  </si>
-  <si>
     <t>line_num_end</t>
   </si>
   <si>
     <t>line_num_start</t>
   </si>
   <si>
-    <t>02619</t>
-  </si>
-  <si>
-    <t>02719</t>
-  </si>
-  <si>
-    <t>02819</t>
-  </si>
-  <si>
-    <t>02919</t>
-  </si>
-  <si>
-    <t>02159</t>
-  </si>
-  <si>
-    <t>02080</t>
-  </si>
-  <si>
-    <t>02099</t>
-  </si>
-  <si>
-    <t>02060</t>
-  </si>
-  <si>
-    <t>02079</t>
-  </si>
-  <si>
-    <t>02180</t>
-  </si>
-  <si>
-    <t>02199</t>
-  </si>
-  <si>
-    <t>02040</t>
-  </si>
-  <si>
-    <t>02059</t>
-  </si>
-  <si>
-    <t>02120</t>
-  </si>
-  <si>
-    <t>02139</t>
-  </si>
-  <si>
     <t>00899</t>
   </si>
   <si>
@@ -521,9 +440,6 @@
     <t>01299</t>
   </si>
   <si>
-    <t>03099</t>
-  </si>
-  <si>
     <t>03599</t>
   </si>
   <si>
@@ -555,12 +471,6 @@
   </si>
   <si>
     <t>name of chain organization</t>
-  </si>
-  <si>
-    <t>S200000</t>
-  </si>
-  <si>
-    <t>04001</t>
   </si>
   <si>
     <t>typ_control</t>
@@ -931,16 +841,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC2BB4DF-E65D-224C-B8BB-1875153B4956}">
-  <dimension ref="A1:G91"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11.1640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.1640625" customWidth="1"/>
-    <col min="7" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="11.1875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1875" customWidth="1"/>
+    <col min="7" max="7" width="7.6875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -951,19 +861,19 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -983,7 +893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1003,7 +913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1023,7 +933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1043,7 +953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1063,7 +973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1083,7 +993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -1103,7 +1013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1123,7 +1033,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
@@ -1143,7 +1053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -1163,7 +1073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -1183,7 +1093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
@@ -1203,7 +1113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
@@ -1223,7 +1133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>31</v>
       </c>
@@ -1243,7 +1153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>33</v>
       </c>
@@ -1263,7 +1173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1283,7 +1193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1303,7 +1213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -1323,7 +1233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
@@ -1343,7 +1253,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -1363,7 +1273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
@@ -1383,7 +1293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
@@ -1403,7 +1313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>45</v>
       </c>
@@ -1423,7 +1333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
@@ -1443,7 +1353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -1463,7 +1373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
@@ -1483,7 +1393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>52</v>
       </c>
@@ -1503,9 +1413,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>46</v>
@@ -1517,7 +1427,7 @@
         <v>49</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="F29">
         <v>10</v>
@@ -1526,9 +1436,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>46</v>
@@ -1537,10 +1447,10 @@
         <v>32</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
       <c r="F30">
         <v>10</v>
@@ -1549,9 +1459,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>46</v>
@@ -1563,7 +1473,7 @@
         <v>21</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -1572,9 +1482,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>46</v>
@@ -1583,10 +1493,10 @@
         <v>32</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>159</v>
+        <v>132</v>
       </c>
       <c r="F32">
         <v>10</v>
@@ -1595,9 +1505,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>46</v>
@@ -1606,10 +1516,10 @@
         <v>32</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="F33">
         <v>10</v>
@@ -1618,7 +1528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
@@ -1638,9 +1548,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>46</v>
@@ -1649,7 +1559,7 @@
         <v>32</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F35">
         <v>10</v>
@@ -1658,9 +1568,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>37</v>
@@ -1669,7 +1579,7 @@
         <v>7</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F36">
         <v>10</v>
@@ -1678,9 +1588,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>37</v>
@@ -1689,7 +1599,7 @@
         <v>7</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F37">
         <v>10</v>
@@ -1698,9 +1608,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A38" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>37</v>
@@ -1709,7 +1619,7 @@
         <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F38">
         <v>10</v>
@@ -1718,9 +1628,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A39" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>37</v>
@@ -1729,7 +1639,7 @@
         <v>6</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F39">
         <v>10</v>
@@ -1738,9 +1648,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A40" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>37</v>
@@ -1749,7 +1659,7 @@
         <v>6</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F40">
         <v>10</v>
@@ -1758,18 +1668,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A41" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F41">
         <v>10</v>
@@ -1778,18 +1688,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A42" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="F42">
         <v>10</v>
@@ -1798,12 +1708,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A43" s="1" t="s">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>32</v>
@@ -1812,7 +1722,7 @@
         <v>44</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
       <c r="F43">
         <v>10</v>
@@ -1821,18 +1731,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A44" s="1" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="F44">
         <v>10</v>
@@ -1841,18 +1751,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A45" s="1" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="B45" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F45">
         <v>10</v>
@@ -1861,12 +1771,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="B46" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>6</v>
@@ -1881,936 +1791,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B47" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="F47">
         <v>10</v>
       </c>
       <c r="G47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F48">
-        <v>96</v>
-      </c>
-      <c r="G48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F49">
-        <v>96</v>
-      </c>
-      <c r="G49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50">
-        <v>96</v>
-      </c>
-      <c r="G50">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F51">
-        <v>96</v>
-      </c>
-      <c r="G51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F52">
-        <v>96</v>
-      </c>
-      <c r="G52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A53" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F53">
-        <v>96</v>
-      </c>
-      <c r="G53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F54">
-        <v>96</v>
-      </c>
-      <c r="G54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F55">
-        <v>96</v>
-      </c>
-      <c r="G55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F56">
-        <v>96</v>
-      </c>
-      <c r="G56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F57">
-        <v>96</v>
-      </c>
-      <c r="G57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A58" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F58">
-        <v>96</v>
-      </c>
-      <c r="G58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A59" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F59">
-        <v>96</v>
-      </c>
-      <c r="G59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A60" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F60">
-        <v>96</v>
-      </c>
-      <c r="G60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F61">
-        <v>96</v>
-      </c>
-      <c r="G61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A62" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F62">
-        <v>96</v>
-      </c>
-      <c r="G62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F63">
-        <v>96</v>
-      </c>
-      <c r="G63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A64" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F64">
-        <v>96</v>
-      </c>
-      <c r="G64">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F65">
-        <v>96</v>
-      </c>
-      <c r="G65">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F66">
-        <v>96</v>
-      </c>
-      <c r="G66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A67" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F67">
-        <v>96</v>
-      </c>
-      <c r="G67">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A68" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F68">
-        <v>96</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A69" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F69">
-        <v>96</v>
-      </c>
-      <c r="G69">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F70">
-        <v>96</v>
-      </c>
-      <c r="G70">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F71">
-        <v>96</v>
-      </c>
-      <c r="G71">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A72" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F72">
-        <v>96</v>
-      </c>
-      <c r="G72">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F73">
-        <v>96</v>
-      </c>
-      <c r="G73">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A74" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="F74">
-        <v>96</v>
-      </c>
-      <c r="G74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A75" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F75">
-        <v>96</v>
-      </c>
-      <c r="G75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A76" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F76">
-        <v>96</v>
-      </c>
-      <c r="G76">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A77" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="E77" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="F77">
-        <v>96</v>
-      </c>
-      <c r="G77">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A78" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="F78">
-        <v>96</v>
-      </c>
-      <c r="G78">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A79" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="F79">
-        <v>96</v>
-      </c>
-      <c r="G79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A80" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="F80">
-        <v>96</v>
-      </c>
-      <c r="G80">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="F81">
-        <v>96</v>
-      </c>
-      <c r="G81">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A82" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F82">
-        <v>96</v>
-      </c>
-      <c r="G82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F83">
-        <v>96</v>
-      </c>
-      <c r="G83">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A84" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F84">
-        <v>96</v>
-      </c>
-      <c r="G84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="F85">
-        <v>96</v>
-      </c>
-      <c r="G85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F86">
-        <v>96</v>
-      </c>
-      <c r="G86">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A87" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="F87">
-        <v>96</v>
-      </c>
-      <c r="G87">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="F88">
-        <v>96</v>
-      </c>
-      <c r="G88">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A89" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B89" t="s">
-        <v>173</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F89">
-        <v>96</v>
-      </c>
-      <c r="G89">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A90" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="B90" t="s">
-        <v>173</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F90">
-        <v>96</v>
-      </c>
-      <c r="G90">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A91" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="B91" t="s">
-        <v>173</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="F91">
-        <v>96</v>
-      </c>
-      <c r="G91">
         <v>1</v>
       </c>
     </row>
@@ -2823,539 +1820,539 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F01AFD1-3AE8-2C43-8863-F91A96C0A348}">
   <dimension ref="A1:C48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="70" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A29" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A30" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" t="s">
         <v>109</v>
       </c>
-      <c r="C28" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A31" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" t="s">
         <v>110</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A32" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" t="s">
         <v>111</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C30" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A33" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" t="s">
         <v>112</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C32" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C33" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C37" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A38" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A39" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A40" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C41" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A42" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A43" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A44" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A45" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C38" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C39" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C41" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C42" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C44" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="B45" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C45" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A46" s="1" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="C46" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A47" s="1" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="C47" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A48" s="1" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="C48" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>